<commit_message>
Implement valve classification enhancements and add support for legend images in hierarchy processing
- Introduced new functions for valve tag identification, stripping prefixes, and inferring valve types based on descriptions.
- Enhanced equipment row building to accommodate valve classifications and reasoning.
- Added command-line options for specifying legend images and output paths for hierarchy CSV and JSON files.
- Updated Makefile to include new targets for valve classification and testing.
- Improved handling of existing outputs and added parallel processing capabilities for hierarchy orchestration.
- Cleaned up comments and organized imports across multiple files for better readability.
</commit_message>
<xml_diff>
--- a/outputs/Broke System.functional_locations.xlsx
+++ b/outputs/Broke System.functional_locations.xlsx
@@ -314,37 +314,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Sinan Aydın</author>
-  </authors>
-  <commentList>
-    <comment ref="A2" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Alanın formatı ve karakter sayısı hakkında bilgi.
-CHAR herhangi bir karakter girilebileceği
-NUM sadece nümerik değer girilebileceği
-DATE tarih formatında alan girilebileceğini,
-gösterir...
-</t>
-      </text>
-    </comment>
-    <comment ref="A5" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Alanın doldurulmasının zorunlu olup, olmadığını gösterir.
-</t>
-      </text>
-    </comment>
-    <comment ref="A6" authorId="0" shapeId="0">
-      <text>
-        <t>Bu alan işaretli olduğunda, alan için değer, seçim kutusundaki değerlerden seçilir.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -646,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:S61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.42578125" customWidth="1" min="1" max="1"/>
@@ -1474,7 +1443,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2005</t>
+          <t>2009</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1598,7 +1567,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2005</t>
+          <t>300</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1679,6 +1648,2776 @@
         </is>
       </c>
       <c r="S16" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24L006</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0060</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>35-24L006 BROKE CVYR 3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24L007</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0070</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>35-24L007 SLABBING PLPR</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24L008</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0080</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>35-24L008 WINDER PLPR</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24L009</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0090</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>35-24L009 BROKE ROLL PLPR</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24L010</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0100</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>35-24L010 BROKE SCRN</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>2031</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24L011</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>35-24L011 BROKE CVYR 1</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P501</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>0120</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>35-24P501 COUCH PIT PMP</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P502</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>0130</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>35-24P502 COUCH PIT PMP</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P503</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>0140</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>35-24P503 PRESS PLPR GRBX OL PMP</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P504</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>0150</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>35-24P504 BROKE CONV 1 PMP</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P505</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>0160</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>35-24P505 SIZE PRESS PLPR PMP</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P506</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>0170</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>35-24P506 REEL PLPR PMP</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P507</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>0180</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>35-24P507 BROKE CONV 3 PMP</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P508</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>0190</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>35-24P508 SLABBING PLPR PMP</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P509</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>0200</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>35-24P509 GB OL PMP</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P510</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>0210</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>35-24P510 BROKE PMP</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P511</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>0220</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>35-24P511 BROKE COLL PMP 60L/S</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P512</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>0230</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>35-24P512 BROKE PMP</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P513</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>0240</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>35-24P513 BR1 BROKE PMP</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P514</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>0250</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>35-24P514 BROKE STOR PMP</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P515</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>0260</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>35-24P515 THICKENED BROKE PMP</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P516</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>0270</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>35-24P516 BROKE FLTRT PMP</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P517</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>0280</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>35-24P517 BROKE DOS PMP</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P518</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>0290</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>35-24P518 BROKE REJ PMP</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P519</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>35-24P519 BROKE ROLL PLPR PMP</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24P520</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>0310</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>35-24P520 REEL PULPR PMP</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24T601</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>0320</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>35-24T601 COUCH PIT TNK 176M3</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>601</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24T602</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>0330</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>35-24T602 BROKE STOR TWR 4000M3</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>601</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24T603</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>0340</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>35-24T603 BROKE COLLECTION TNK 40M3</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>601</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24T604</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>0350</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>35-24T604 BROKE FLTRT TNK 40M3</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>601</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24T605</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>0360</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>35-24T605 THICKENED BROKE TNK 70M3</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>601</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24T606</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>0370</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>35-24T606 BROKE REJ TNK 15M3</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>601</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24T607</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>0380</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>35-24T607 BROKE DOS TNK 35M3</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>601</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24ES-508</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>0390</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>35-24ES-508 WINDER AREA EMERG STOP</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>1108</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24ES-601</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>35-24ES-601 UTM E-STOP</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>1108</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24ES-662</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>0410</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>35-24ES-662 BROKE THICKENER EMRG STOP</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>1108</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24ES-663</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>0420</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>35-24ES-663 BROKE THICKENER E-STOP</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>1108</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24ES-683</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>0430</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>35-24ES-683 BROK ROLL PLPR EMRG STOP</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>1108</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>ELEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24HI-501</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>0440</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>35-24HI-501 HI VLV POSITION IND</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>201</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24HI-503</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>0450</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>35-24HI-503 WNDR PLPR SHW S5 S6 IND</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24HI-516</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>0460</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>35-24HI-516 WNDR PLPR SHW S1 S2 IND</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24HI-529</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>0470</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>35-24HI-529 SLBG PLPR SHW S1 IND</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24HI-532</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>0480</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>35-24HI-532 HIGH IND INSTR</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24HI-534</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>0490</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>35-24HI-534 HIGH IND</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1-35-24HI-552</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>5001-PM03-BR-BR1</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>NNNN-XXXX-AA-XXX-XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>35-24HI-552 REEL PLPR TAIL SHW ST IND</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>5001</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
         <is>
           <t>MECH</t>
         </is>
@@ -1694,6 +4433,5 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Enhance valve classification and hierarchy processing
- Added support for orphan valve rows in hierarchy to prevent loss of P-VALVEPOS tags without nearby FUNCTION nodes.
- Updated bowtie fill rules in `dwg_valve_classify.py` for improved classification accuracy.
- Introduced new functions for grouping tags by input and loading drawing context in `test_valve_cad_vision_cases.py`.
- Adjusted expected types in test cases to include new valve classifications.
- Cleaned up and organized code for better readability and maintainability across multiple files.
</commit_message>
<xml_diff>
--- a/outputs/Broke System.functional_locations.xlsx
+++ b/outputs/Broke System.functional_locations.xlsx
@@ -2792,7 +2792,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>35-24P513 BR1 BROKE PMP</t>
+          <t>35-24P513 BR1 BROKE PMP 140L/S</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2854,7 +2854,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>35-24P514 BROKE STOR PMP</t>
+          <t>35-24P514 BROKE STOR TWR PMP</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>35-24T602 BROKE STOR TWR TNK</t>
+          <t>35-24T602 BROKE STOR TWR 4000M3</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>35-24HI-501 HI HND IND</t>
+          <t>35-24HI-501 HI VLV POSITION IND</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -4045,6 +4045,11 @@
           <t>M</t>
         </is>
       </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>201</t>
+        </is>
+      </c>
       <c r="O55" t="inlineStr">
         <is>
           <t>5001</t>
@@ -4058,6 +4063,11 @@
       <c r="R55" t="inlineStr">
         <is>
           <t>P01</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>MECH</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4094,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>35-24HI-503 WNDR PLPR SHW S5 S6 IND</t>
+          <t>35-24HI-503 WNDR PLPR SHW S5&amp;S6 IND</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -4208,7 +4218,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>35-24HI-529 SLABBING PLPR SHW S1</t>
+          <t>35-24HI-529 SLABBING PLPR SHW S1 IND</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -4270,7 +4280,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>35-24HI-532 HIGH IND INSTR</t>
+          <t>35-24HI-532 HIGH IND</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -4436,7 +4446,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>35-24HI-555 REEL PLPR SHW S1 IND</t>
+          <t>35-24HI-555 REEL PLPR SHW S1 HI</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -4498,7 +4508,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>35-24HI-572 HI WAF LVL IND</t>
+          <t>35-24HI-572 LVL HI INSTR</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -4550,7 +4560,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>35-24HI-575 HIGH IND</t>
+          <t>35-24HI-575 HIGH IND INSTR</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -4912,7 +4922,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>35-24HI-652 HIGH IND</t>
+          <t>35-24HI-652 HIGH IND INST</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -5088,7 +5098,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>35-24HS-501 HS BROKE DIL VLV CTRL</t>
+          <t>35-24HS-501 HND SW</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -5101,11 +5111,6 @@
           <t>M</t>
         </is>
       </c>
-      <c r="N73" t="inlineStr">
-        <is>
-          <t>202</t>
-        </is>
-      </c>
       <c r="O73" t="inlineStr">
         <is>
           <t>5001</t>
@@ -5119,11 +5124,6 @@
       <c r="R73" t="inlineStr">
         <is>
           <t>P01</t>
-        </is>
-      </c>
-      <c r="S73" t="inlineStr">
-        <is>
-          <t>MECH</t>
         </is>
       </c>
     </row>
@@ -5398,7 +5398,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>35-24HS-529 SLABBING PLPR SHW S1 HS</t>
+          <t>35-24HS-529 SLBNG PLPR SHW S1 HS</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -5460,7 +5460,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>35-24HS-532 HS SELECTOR SW</t>
+          <t>35-24HS-532 HND SW</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -5698,7 +5698,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>35-24HS-555 HND SW BROKE SEL</t>
+          <t>35-24HS-555 HND SW</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -5874,7 +5874,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>35-24HS-575 HND SW</t>
+          <t>35-24HS-575 HND SW BROKE CONV 2</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -5988,7 +5988,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>35-24HS-583 HND SW</t>
+          <t>35-24HS-583 HND SW BROKE DIST</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>35-24HS-629 BROKE THKR LOC/REMOTE SW</t>
+          <t>35-24HS-629 LOC/REMOTE SEL SW</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -6392,7 +6392,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>35-24HS-652 HND SW STN</t>
+          <t>35-24HS-652 HND SW</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -6568,7 +6568,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>35-24HS-664 COUCH PIT START STOP</t>
+          <t>35-24HS-664 COUCH PIT START STOP HS</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -6620,7 +6620,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>35-24HS-682 BROK ROLL PLPR START/STOP</t>
+          <t>35-24HS-682 BROK ROLL PLPR START STOP</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -6682,7 +6682,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>35-24KJ-510 WINDER PLPR START PB</t>
+          <t>35-24KJ-510 WINDER PLPR START</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -6744,7 +6744,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>35-24KJ-511 WNDR PLPR STOP PUSHBTN</t>
+          <t>35-24KJ-511 WNDR PLPR STOP</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>35-24KJ-544 REEL PULPR STOP</t>
+          <t>35-24KJ-544 REEL PLPR STOP</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -7005,6 +7005,11 @@
           <t>M</t>
         </is>
       </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
       <c r="O105" t="inlineStr">
         <is>
           <t>5001</t>
@@ -7018,6 +7023,11 @@
       <c r="R105" t="inlineStr">
         <is>
           <t>P01</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>MECH</t>
         </is>
       </c>
     </row>
@@ -7624,7 +7634,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>35-24KJ-688 BROKE SCRN START SEQ</t>
+          <t>35-24KJ-688 BROKE SCRNG START SEQ</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -7686,7 +7696,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>35-24KJ-689 BROKE SCRNG STOP SEQ</t>
+          <t>35-24KJ-689 BROKE SCRN STOP SEQ</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -8058,7 +8068,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>35-24XS-691 WNDR AREA MCS SIG</t>
+          <t>35-24XS-691 WNDR PLPR MCS SIGNAL</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -8182,7 +8192,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>35-24-008 WINDER PLPR WFL LN</t>
+          <t>35-24-008 WFL LN WINDER PLPR</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -8306,7 +8316,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>35-24-012 WFL 15 PROC LN</t>
+          <t>35-24-012 WFL-15 PROC LN</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -8358,7 +8368,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>35-24-016 WAF 250 HEADER LN</t>
+          <t>35-24-016 WAF 250 DIST HDR</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -8410,7 +8420,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>35-24-017 WAF 300 LN</t>
+          <t>35-24-017 WAF LN DN300</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -8514,7 +8524,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>35-24-026 WFL 15 GB OL LUB LN</t>
+          <t>35-24-026 WFL 15 GB OL FLSH LN</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -8722,7 +8732,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>35-24-042 WFL LN DN15</t>
+          <t>35-24-042 WFL LN</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -8930,7 +8940,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>35-24-052 WAF 300 DIST HDR LN</t>
+          <t>35-24-052 WAF 300 BROKE DIST HDR</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -9034,7 +9044,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>35-24-056 WAF-350 BROKE HDR LN</t>
+          <t>35-24-056 WAF-350 BROKE LN</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -9086,7 +9096,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>35-24-061 WFL 15 PROC LN</t>
+          <t>35-24-061 WFL LN DN15</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -9138,7 +9148,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>35-24-063 WAF-250 BROKE LN</t>
+          <t>35-24-063 WAF 250 BROKE LN</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -9190,7 +9200,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>35-24-068 WFL LN DN15</t>
+          <t>35-24-068 WFL LN BR1</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -9242,7 +9252,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>35-24-076 WFL LN 15 GB OL</t>
+          <t>35-24-076 WFL 15 GB OL FL LN</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -9294,7 +9304,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>35-24-079 WFL 15 FL LN</t>
+          <t>35-24-079 WFL LN DN15</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -9346,7 +9356,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>35-24-080 WFL LN</t>
+          <t>35-24-080 WFL LN 15</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -9554,7 +9564,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>35-24-089 WAF-300 LN</t>
+          <t>35-24-089 WAF LN DN300</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -9658,7 +9668,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>35-24-098 WAF LN 300</t>
+          <t>35-24-098 WAF-300 PROC LN</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
@@ -9866,7 +9876,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>35-24-105 WAF-300 PROC LN</t>
+          <t>35-24-105 WAF LN BR1 SHW</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -9879,6 +9889,11 @@
           <t>M</t>
         </is>
       </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
       <c r="O157" t="inlineStr">
         <is>
           <t>5001</t>
@@ -9892,6 +9907,11 @@
       <c r="R157" t="inlineStr">
         <is>
           <t>P01</t>
+        </is>
+      </c>
+      <c r="S157" t="inlineStr">
+        <is>
+          <t>MECH</t>
         </is>
       </c>
     </row>
@@ -9970,7 +9990,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>35-24-109 WAF 500 LN</t>
+          <t>35-24-109 WAF 500 BROKE LN</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -10022,7 +10042,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>35-24-112 WAF-400 APPROACH FL LN</t>
+          <t>35-24-112 WAF-400 PROC LN</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -10230,7 +10250,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>35-24-122 WFL LN BR1</t>
+          <t>35-24-122 WFL SHW LN DN15</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
@@ -10243,6 +10263,11 @@
           <t>M</t>
         </is>
       </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
       <c r="O164" t="inlineStr">
         <is>
           <t>5001</t>
@@ -10256,6 +10281,11 @@
       <c r="R164" t="inlineStr">
         <is>
           <t>P01</t>
+        </is>
+      </c>
+      <c r="S164" t="inlineStr">
+        <is>
+          <t>MECH</t>
         </is>
       </c>
     </row>
@@ -10282,7 +10312,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>35-24-123 WFL PROC LN DN15</t>
+          <t>35-24-123 WFL PROC LN</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -10542,7 +10572,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>35-24-138 WFL LN</t>
+          <t>35-24-138 WFL 15 FLSH LN</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
@@ -10698,7 +10728,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>35-24-160 WFL PROC LN</t>
+          <t>35-24-160 WFL LN BR1</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -10750,7 +10780,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>35-24-163 WFL LN DN15</t>
+          <t>35-24-163 WFL 15 PROC LN</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -10802,7 +10832,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>35-24-167 PROC LN WFL DN15</t>
+          <t>35-24-167 BROKE PROC LN</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
@@ -10958,7 +10988,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>35-24-185 WAF 150 LN</t>
+          <t>35-24-185 WAF 150 BROKE LN</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
@@ -11062,7 +11092,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>35-24-195 WFL LN</t>
+          <t>35-24-195 WFL LN DN15</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -11270,7 +11300,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>35-24-216 CLG WTR RTN LN</t>
+          <t>35-24-216 COOL WTR RTN LN</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
@@ -11322,7 +11352,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>35-24-219 WFL LN DN15</t>
+          <t>35-24-219 WFL LN 15</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
@@ -11374,7 +11404,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>35-24-224 WFL LN BR1</t>
+          <t>35-24-224 WFL LN DN15</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
@@ -11478,7 +11508,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>35-25-072 WAF LN DN350 FM WHT WTR TNK</t>
+          <t>35-25-072 WAF LN DN350</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -11491,11 +11521,6 @@
           <t>M</t>
         </is>
       </c>
-      <c r="N188" t="inlineStr">
-        <is>
-          <t>601</t>
-        </is>
-      </c>
       <c r="O188" t="inlineStr">
         <is>
           <t>5001</t>
@@ -11509,11 +11534,6 @@
       <c r="R188" t="inlineStr">
         <is>
           <t>P01</t>
-        </is>
-      </c>
-      <c r="S188" t="inlineStr">
-        <is>
-          <t>MECH</t>
         </is>
       </c>
     </row>

</xml_diff>